<commit_message>
feat(M1): 经济底座 save v2 + type5/6/7 + debug_panel  M1 里程碑完成： - save_manager v2（save_version=2，三货币/intellevel/fanlevel/inventory/feed_instances） - EconomyManager + ConditionChecker type5/6/7 - debug_panel（F12 开发入口） - 配表：banner_config、levels grant*、艺人帖 condition_id=4、教程种子帖 9001 - economy_test / flow_test / loop_test 全过
修复 cleanup_debug_logs 误删：
- idol_popup_panel Z_INDEX_* / BUBBLE_DISMISS_CANVAS_LAYER 常量恢复
- feed_post_card 删除 debug_log_card_layout 残留调用
- ui_router 移除临时活动/商城按钮

设计说明：新档 intellevel=0 时艺人 Tab 空列表为 type5 预期行为。
M2 待做：通关 grant 发奖、ExposeManager 玩家流、Fanclub 正式 UI（M4）。
</commit_message>
<xml_diff>
--- a/data_src/xlsx表/商城上架表.xlsx
+++ b/data_src/xlsx表/商城上架表.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,45 +424,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>currencytype</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>itemid</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>shopdesc</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>shopicon</t>
+          <t>conditionid</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>conditionid</t>
+          <t>stocklimit</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>stocklimit</t>
+          <t>shoptab</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>shoptab</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
         <is>
           <t>tutorialonly</t>
         </is>
@@ -471,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,12 +486,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -510,11 +505,6 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -523,53 +513,79 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>上架 id</t>
+          <t>上架id</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22饭圈积分/23星星/24情报点</t>
+          <t>名称</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>售价</t>
+          <t>货币类型</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>购买后给的道具</t>
+          <t>价格</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>商城展示描述</t>
+          <t>道具id</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>art/icons 展示图</t>
+          <t>条件id</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>显示条件；0=无条件</t>
+          <t>库存上限</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-1=无限</t>
+          <t>商城页签</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1周边售卖/2周边兑换</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0/1</t>
-        </is>
+          <t>教程专用</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>教程专辑</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>